<commit_message>
better formatting of config templates
</commit_message>
<xml_diff>
--- a/src/cassy/additional_data/templates/bolts/Flange1.xlsx
+++ b/src/cassy/additional_data/templates/bolts/Flange1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\runners\bolts\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laghida\Documents\Github\cassy\src\cassy\additional_data\templates\bolts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3432AB52-13CB-43EC-8D8F-5F85BB0696C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA08ABCC-80ED-4158-8F97-9CD6513D1ADE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REs" sheetId="1" r:id="rId1"/>
@@ -222,15 +222,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.14999847407452621"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="12">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -238,188 +250,40 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -704,531 +568,531 @@
   <dimension ref="A1:K15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="11" width="13.7109375" customWidth="1"/>
+    <col min="1" max="11" width="16.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="3" t="s">
+      <c r="K1" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" s="11">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="13">
-        <v>35</v>
-      </c>
-      <c r="G2" s="13">
-        <v>0</v>
-      </c>
-      <c r="H2" s="12" t="s">
+      <c r="C2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="7">
+        <v>35</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+      <c r="H2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="14" t="s">
+      <c r="J2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="16">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5">
-        <v>35</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0</v>
-      </c>
-      <c r="H3" s="4" t="s">
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7">
+        <v>35</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0</v>
+      </c>
+      <c r="H3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J3" s="4" t="s">
+      <c r="J3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="16">
+      <c r="A4" s="9">
         <v>1</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5">
-        <v>35</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0</v>
-      </c>
-      <c r="H4" s="4" t="s">
+      <c r="E4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="7">
+        <v>35</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="J4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K4" s="17" t="s">
+      <c r="K4" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="16">
+      <c r="A5" s="9">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="4" t="s">
+      <c r="C5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="5">
+      <c r="E5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="7">
         <v>145</v>
       </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5" s="4" t="s">
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="4" t="s">
+      <c r="J5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="16">
+      <c r="A6" s="9">
         <v>1</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="5">
-        <v>35</v>
-      </c>
-      <c r="G6" s="5">
-        <v>0</v>
-      </c>
-      <c r="H6" s="4" t="s">
+      <c r="E6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="7">
+        <v>35</v>
+      </c>
+      <c r="G6" s="7">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="J6" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="16">
+      <c r="A7" s="9">
         <v>1</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="5">
+      <c r="F7" s="7">
         <v>300</v>
       </c>
-      <c r="G7" s="5">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4" t="s">
+      <c r="G7" s="7">
+        <v>0</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="J7" s="4" t="s">
+      <c r="J7" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="18">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="9">
         <v>1</v>
       </c>
-      <c r="B8" s="19" t="s">
+      <c r="B8" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="19" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" s="19" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="21">
-        <v>35</v>
-      </c>
-      <c r="G8" s="21">
-        <v>0</v>
-      </c>
-      <c r="H8" s="22" t="s">
+      <c r="C8" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="7">
+        <v>35</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="22" t="s">
+      <c r="J8" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K8" s="23" t="s">
+      <c r="K8" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="9">
         <v>2</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" s="5">
-        <v>35</v>
-      </c>
-      <c r="G9" s="5">
-        <v>0</v>
-      </c>
-      <c r="H9" s="12" t="s">
+      <c r="C9" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" s="7">
+        <v>35</v>
+      </c>
+      <c r="G9" s="7">
+        <v>0</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="6" t="s">
+      <c r="J9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="6" t="s">
+      <c r="K9" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="9">
         <v>2</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" s="5">
-        <v>35</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4" t="s">
+      <c r="E10" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="7">
+        <v>35</v>
+      </c>
+      <c r="G10" s="7">
+        <v>0</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="I10" s="4" t="s">
+      <c r="I10" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J10" s="4" t="s">
+      <c r="J10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="K10" s="4" t="s">
+      <c r="K10" s="6" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="9">
         <v>2</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="5">
-        <v>35</v>
-      </c>
-      <c r="G11" s="5">
-        <v>0</v>
-      </c>
-      <c r="H11" s="4" t="s">
+      <c r="E11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="7">
+        <v>35</v>
+      </c>
+      <c r="G11" s="7">
+        <v>0</v>
+      </c>
+      <c r="H11" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="I11" s="4" t="s">
+      <c r="I11" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="J11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K11" s="4" t="s">
+      <c r="K11" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="9">
         <v>2</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C12" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" s="5">
+      <c r="E12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="7">
         <v>145</v>
       </c>
-      <c r="G12" s="5">
-        <v>0</v>
-      </c>
-      <c r="H12" s="4" t="s">
+      <c r="G12" s="7">
+        <v>0</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I12" s="4" t="s">
+      <c r="I12" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="J12" s="4" t="s">
+      <c r="J12" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="K12" s="4" t="s">
+      <c r="K12" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="A13" s="9">
         <v>2</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" s="5">
-        <v>35</v>
-      </c>
-      <c r="G13" s="5">
-        <v>0</v>
-      </c>
-      <c r="H13" s="4" t="s">
+      <c r="E13" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="7">
+        <v>35</v>
+      </c>
+      <c r="G13" s="7">
+        <v>0</v>
+      </c>
+      <c r="H13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I13" s="4" t="s">
+      <c r="I13" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="J13" s="4" t="s">
+      <c r="J13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K13" s="4" t="s">
+      <c r="K13" s="6" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="A14" s="9">
         <v>2</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C14" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C14" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E14" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F14" s="5">
+      <c r="F14" s="7">
         <v>300</v>
       </c>
-      <c r="G14" s="5">
-        <v>0</v>
-      </c>
-      <c r="H14" s="4" t="s">
+      <c r="G14" s="7">
+        <v>0</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I14" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K14" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="9">
         <v>2</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="5">
-        <v>35</v>
-      </c>
-      <c r="G15" s="5">
-        <v>0</v>
-      </c>
-      <c r="H15" s="22" t="s">
+      <c r="C15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="7">
+        <v>35</v>
+      </c>
+      <c r="G15" s="7">
+        <v>0</v>
+      </c>
+      <c r="H15" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="I15" s="22" t="s">
+      <c r="I15" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="J15" s="6" t="s">
+      <c r="J15" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="K15" s="8" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1242,211 +1106,212 @@
   <dimension ref="A1:M5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="13" width="15.7109375" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1"/>
+    <col min="2" max="13" width="15.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="2" t="s">
+      <c r="B1" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="11" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="5">
-        <v>35</v>
-      </c>
-      <c r="G2" s="5">
-        <v>0</v>
-      </c>
-      <c r="H2">
+      <c r="C2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="7">
+        <v>35</v>
+      </c>
+      <c r="G2" s="7">
+        <v>0</v>
+      </c>
+      <c r="H2" s="9">
         <v>1000</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="I2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="L2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" s="5">
-        <v>35</v>
-      </c>
-      <c r="G3" s="5">
-        <v>0</v>
-      </c>
-      <c r="H3">
+      <c r="C3" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="7">
+        <v>35</v>
+      </c>
+      <c r="G3" s="7">
+        <v>0</v>
+      </c>
+      <c r="H3" s="9">
         <v>10</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L3" s="24" t="s">
+      <c r="L3" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M3" s="24" t="s">
+      <c r="M3" s="9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="9">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="5">
-        <v>35</v>
-      </c>
-      <c r="G4" s="5">
-        <v>0</v>
-      </c>
-      <c r="H4">
+      <c r="C4" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="7">
+        <v>35</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="9">
         <v>1000</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="I4" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="6" t="s">
+      <c r="L4" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="M4" s="6" t="s">
+      <c r="M4" s="8" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="9">
         <v>2</v>
       </c>
-      <c r="B5" s="24" t="s">
+      <c r="B5" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="C5" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="5">
-        <v>35</v>
-      </c>
-      <c r="G5" s="5">
-        <v>0</v>
-      </c>
-      <c r="H5">
+      <c r="C5" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="7">
+        <v>35</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+      <c r="H5" s="9">
         <v>10</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="L5" s="24" t="s">
+      <c r="L5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M5" s="24" t="s">
+      <c r="M5" s="9" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1460,78 +1325,76 @@
   <dimension ref="A1:D5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" customWidth="1"/>
-    <col min="4" max="4" width="11" customWidth="1"/>
+    <col min="1" max="4" width="13.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="7">
+      <c r="D2" s="4">
         <v>200000</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="7">
+      <c r="D3" s="4">
         <v>200000</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D4" s="7">
+      <c r="D4" s="4">
         <v>200000</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="1">
         <v>2</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D5" s="7">
+      <c r="D5" s="4">
         <v>200000</v>
       </c>
     </row>
@@ -1550,10 +1413,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="2" t="s">
         <v>47</v>
       </c>
     </row>
@@ -1561,7 +1424,7 @@
       <c r="A2" t="s">
         <v>45</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="3" t="s">
         <v>56</v>
       </c>
     </row>

</xml_diff>